<commit_message>
docs: consolida inventário com status real da coleta de PANs
Atualiza status da fonte PANs (F002) para refletir os 74 PANs mapeados e
985 documentos baixados, e adiciona aba detalhando os 7 PANs de
herpetofauna (foco temático do projeto), todos pendentes de classificação
de sensibilidade antes de qualquer indexação.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/06_inventario/inventario_fontes.xlsx
+++ b/06_inventario/inventario_fontes.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes gerais" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publicações científicas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PANs - Herpetofauna" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes gerais'!$A$1:$J$6</definedName>
@@ -599,7 +600,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A mapear</t>
+          <t>Coletado — metadados de 74 PANs mapeados (01_fontes_web/pans/_indice_pans.json); 985 documentos (PDF/XLSX) baixados. Pendente: classificação de sensibilidade antes de mover para 03_documentos_autorizados/04_documentos_pendentes_avaliacao.</t>
         </is>
       </c>
     </row>
@@ -1016,4 +1017,326 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status do PAN</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Documentos listados</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Documentos baixados</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Caminho local</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sensibilidade</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Status de classificação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pan-herpetofauna-do-nordeste</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Herpetofauna do Nordeste</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>em_execucao</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-herpetofauna-do-nordeste/documentos/</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pan-herpetofauna-do-sudeste</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Herpetofauna do Sudeste</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>em_execucao</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-herpetofauna-do-sudeste/documentos/</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pan-herpetofauna-do-sul</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Herpetofauna do Sul</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>em_execucao</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-herpetofauna-do-sul/documentos/</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pan-herpetofauna-do-espinhaco</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Herpetofauna do Espinhaço</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>finalizado</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-herpetofauna-do-espinhaco/documentos/</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pan-herpetofauna-insular</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Herpetofauna Insular</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>finalizado</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-herpetofauna-insular/documentos/</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pan-quelonios</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Quelônios</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>finalizado</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-quelonios/documentos/</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>pan-tartarugas-marinhas</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tartarugas Marinhas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>em_execucao</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E8" t="n">
+        <v>17</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>01_fontes_web/pans/pan-tartarugas-marinhas/documentos/</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A avaliar</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pendente avaliação</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona textos autorizados de Monitora/PANs e registro de classificação
Copia os textos extraídos de Monitora e PANs para 03_documentos_autorizados/
(fontes públicas, conforme ADR 0002), habilitando o chunking já executado
dessas fontes (Fase 4.2). Adiciona o registro de classificação de
sensibilidade (06_inventario/classificacao_monitora_pans_salve_2026-07-03.json)
e atualiza o inventário consolidado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/06_inventario/inventario_fontes.xlsx
+++ b/06_inventario/inventario_fontes.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A mapear</t>
+          <t>Classificado em 2026-07-03: 109/109 documentos extraídos autorizados (zero coordenada precisa de espécie/dado pessoal detectado). Copiados para 03_documentos_autorizados/monitora/. Ver 06_inventario/classificacao_monitora_pans_salve_2026-07-03.json</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Público</t>
+          <t>Público (7 documentos com dado pessoal tratados à parte)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Coletado — metadados de 74 PANs mapeados (01_fontes_web/pans/_indice_pans.json); 985 documentos (PDF/XLSX) baixados. Pendente: classificação de sensibilidade antes de mover para 03_documentos_autorizados/04_documentos_pendentes_avaliacao.</t>
+          <t>Classificado em 2026-07-03: 706/707 documentos extraídos autorizados (700 diretos + 6 com redação de página para remover CPF de terceiros sem relação com o conteúdo do PAN). 1 documento (pan-quelonios-portaria-gat) classificado como sensível — só contém nomeação de pessoas físicas, sem conteúdo técnico residual, movido para 05_documentos_sensiveis_nao_indexar/. Ver 06_inventario/classificacao_monitora_pans_salve_2026-07-03.json</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>A avaliar</t>
+          <t>Público</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A avaliar</t>
+          <t>Classificado em 2026-07-03: 24/24 fichas extraídas autorizadas — distribuição geográfica só em nível de estado/bioma/bacia hidrográfica, sem coordenada precisa nem dado pessoal. Copiadas para 03_documentos_autorizados/salve/. Ver 06_inventario/classificacao_monitora_pans_salve_2026-07-03.json</t>
         </is>
       </c>
     </row>

</xml_diff>